<commit_message>
Add formula total row to sample and skip total rows when reading
Each line sheet in the sample now ends with a TỔNG / 合计 row: SUM for the
quantity columns, and day/month % computed as total actual / total target.
The reader ignores such total rows (TỔNG, TỔNG CỘNG, Total, 合计, 总计, 小计)
so they are never counted as a product.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ExBHMp87VhZ8YLQXVqanNX
</commit_message>
<xml_diff>
--- a/samples/SanLuong-khach-mau.xlsx
+++ b/samples/SanLuong-khach-mau.xlsx
@@ -72,6 +72,9 @@
     <x:t>BAO TAY XANH</x:t>
   </x:si>
   <x:si>
+    <x:t>TỔNG / 合计</x:t>
+  </x:si>
+  <x:si>
     <x:t>GĂNG TAY TRẮNG</x:t>
   </x:si>
   <x:si>
@@ -88,7 +91,7 @@
     <x:numFmt numFmtId="164" formatCode="#,##0"/>
     <x:numFmt numFmtId="165" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="1">
+  <x:fonts count="2">
     <x:font>
       <x:vertAlign val="baseline"/>
       <x:sz val="11"/>
@@ -96,13 +99,26 @@
       <x:name val="Calibri"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:vertAlign val="baseline"/>
+      <x:sz val="11"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Calibri"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="2">
+  <x:fills count="3">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
     </x:fill>
   </x:fills>
   <x:borders count="2">
@@ -141,7 +157,7 @@
       </x:diagonal>
     </x:border>
   </x:borders>
-  <x:cellStyleXfs count="4">
+  <x:cellStyleXfs count="7">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -154,8 +170,17 @@
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="1" fillId="2" borderId="1" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="6">
+  <x:cellXfs count="9">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -177,6 +202,18 @@
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <x:protection locked="1" hidden="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
@@ -475,7 +512,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K7"/>
+  <x:dimension ref="A1:K8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -619,16 +656,32 @@
       <x:c r="K5" s="3"/>
     </x:row>
     <x:row r="6" spans="1:11">
-      <x:c r="A6" s="3"/>
-      <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-      <x:c r="F6" s="3"/>
-      <x:c r="G6" s="3"/>
-      <x:c r="H6" s="3"/>
-      <x:c r="I6" s="3"/>
-      <x:c r="J6" s="3"/>
+      <x:c r="A6" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="6"/>
+      <x:c r="C6" s="6"/>
+      <x:c r="D6" s="7">
+        <x:f>SUM(D3:D5)</x:f>
+      </x:c>
+      <x:c r="E6" s="7">
+        <x:f>SUM(E3:E5)</x:f>
+      </x:c>
+      <x:c r="F6" s="8">
+        <x:f>IF(D6=0,"",E6/D6)</x:f>
+      </x:c>
+      <x:c r="G6" s="7">
+        <x:f>SUM(G3:G5)</x:f>
+      </x:c>
+      <x:c r="H6" s="7">
+        <x:f>SUM(H3:H5)</x:f>
+      </x:c>
+      <x:c r="I6" s="7">
+        <x:f>SUM(I3:I5)</x:f>
+      </x:c>
+      <x:c r="J6" s="8">
+        <x:f>IF(G6=0,"",H6/G6)</x:f>
+      </x:c>
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -643,6 +696,19 @@
       <x:c r="I7" s="3"/>
       <x:c r="J7" s="3"/>
       <x:c r="K7" s="3"/>
+    </x:row>
+    <x:row r="8" spans="1:11">
+      <x:c r="A8" s="3"/>
+      <x:c r="B8" s="3"/>
+      <x:c r="C8" s="3"/>
+      <x:c r="D8" s="3"/>
+      <x:c r="E8" s="3"/>
+      <x:c r="F8" s="3"/>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3"/>
+      <x:c r="I8" s="3"/>
+      <x:c r="J8" s="3"/>
+      <x:c r="K8" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -661,7 +727,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K7"/>
+  <x:dimension ref="A1:K8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -805,16 +871,32 @@
       <x:c r="K5" s="3"/>
     </x:row>
     <x:row r="6" spans="1:11">
-      <x:c r="A6" s="3"/>
-      <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-      <x:c r="F6" s="3"/>
-      <x:c r="G6" s="3"/>
-      <x:c r="H6" s="3"/>
-      <x:c r="I6" s="3"/>
-      <x:c r="J6" s="3"/>
+      <x:c r="A6" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="6"/>
+      <x:c r="C6" s="6"/>
+      <x:c r="D6" s="7">
+        <x:f>SUM(D3:D5)</x:f>
+      </x:c>
+      <x:c r="E6" s="7">
+        <x:f>SUM(E3:E5)</x:f>
+      </x:c>
+      <x:c r="F6" s="8">
+        <x:f>IF(D6=0,"",E6/D6)</x:f>
+      </x:c>
+      <x:c r="G6" s="7">
+        <x:f>SUM(G3:G5)</x:f>
+      </x:c>
+      <x:c r="H6" s="7">
+        <x:f>SUM(H3:H5)</x:f>
+      </x:c>
+      <x:c r="I6" s="7">
+        <x:f>SUM(I3:I5)</x:f>
+      </x:c>
+      <x:c r="J6" s="8">
+        <x:f>IF(G6=0,"",H6/G6)</x:f>
+      </x:c>
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -829,6 +911,19 @@
       <x:c r="I7" s="3"/>
       <x:c r="J7" s="3"/>
       <x:c r="K7" s="3"/>
+    </x:row>
+    <x:row r="8" spans="1:11">
+      <x:c r="A8" s="3"/>
+      <x:c r="B8" s="3"/>
+      <x:c r="C8" s="3"/>
+      <x:c r="D8" s="3"/>
+      <x:c r="E8" s="3"/>
+      <x:c r="F8" s="3"/>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3"/>
+      <x:c r="I8" s="3"/>
+      <x:c r="J8" s="3"/>
+      <x:c r="K8" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -847,7 +942,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K8"/>
+  <x:dimension ref="A1:K9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -1024,16 +1119,32 @@
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
-      <x:c r="A7" s="3"/>
-      <x:c r="B7" s="3"/>
-      <x:c r="C7" s="3"/>
-      <x:c r="D7" s="3"/>
-      <x:c r="E7" s="3"/>
-      <x:c r="F7" s="3"/>
-      <x:c r="G7" s="3"/>
-      <x:c r="H7" s="3"/>
-      <x:c r="I7" s="3"/>
-      <x:c r="J7" s="3"/>
+      <x:c r="A7" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B7" s="6"/>
+      <x:c r="C7" s="6"/>
+      <x:c r="D7" s="7">
+        <x:f>SUM(D3:D6)</x:f>
+      </x:c>
+      <x:c r="E7" s="7">
+        <x:f>SUM(E3:E6)</x:f>
+      </x:c>
+      <x:c r="F7" s="8">
+        <x:f>IF(D7=0,"",E7/D7)</x:f>
+      </x:c>
+      <x:c r="G7" s="7">
+        <x:f>SUM(G3:G6)</x:f>
+      </x:c>
+      <x:c r="H7" s="7">
+        <x:f>SUM(H3:H6)</x:f>
+      </x:c>
+      <x:c r="I7" s="7">
+        <x:f>SUM(I3:I6)</x:f>
+      </x:c>
+      <x:c r="J7" s="8">
+        <x:f>IF(G7=0,"",H7/G7)</x:f>
+      </x:c>
       <x:c r="K7" s="3"/>
     </x:row>
     <x:row r="8" spans="1:11">
@@ -1048,6 +1159,19 @@
       <x:c r="I8" s="3"/>
       <x:c r="J8" s="3"/>
       <x:c r="K8" s="3"/>
+    </x:row>
+    <x:row r="9" spans="1:11">
+      <x:c r="A9" s="3"/>
+      <x:c r="B9" s="3"/>
+      <x:c r="C9" s="3"/>
+      <x:c r="D9" s="3"/>
+      <x:c r="E9" s="3"/>
+      <x:c r="F9" s="3"/>
+      <x:c r="G9" s="3"/>
+      <x:c r="H9" s="3"/>
+      <x:c r="I9" s="3"/>
+      <x:c r="J9" s="3"/>
+      <x:c r="K9" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -1066,7 +1190,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K7"/>
+  <x:dimension ref="A1:K8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -1112,7 +1236,7 @@
     </x:row>
     <x:row r="3" spans="1:11">
       <x:c r="A3" s="3" t="s">
-        <x:v>13</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="3">
         <x:v>10</x:v>
@@ -1210,16 +1334,32 @@
       <x:c r="K5" s="3"/>
     </x:row>
     <x:row r="6" spans="1:11">
-      <x:c r="A6" s="3"/>
-      <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-      <x:c r="F6" s="3"/>
-      <x:c r="G6" s="3"/>
-      <x:c r="H6" s="3"/>
-      <x:c r="I6" s="3"/>
-      <x:c r="J6" s="3"/>
+      <x:c r="A6" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="6"/>
+      <x:c r="C6" s="6"/>
+      <x:c r="D6" s="7">
+        <x:f>SUM(D3:D5)</x:f>
+      </x:c>
+      <x:c r="E6" s="7">
+        <x:f>SUM(E3:E5)</x:f>
+      </x:c>
+      <x:c r="F6" s="8">
+        <x:f>IF(D6=0,"",E6/D6)</x:f>
+      </x:c>
+      <x:c r="G6" s="7">
+        <x:f>SUM(G3:G5)</x:f>
+      </x:c>
+      <x:c r="H6" s="7">
+        <x:f>SUM(H3:H5)</x:f>
+      </x:c>
+      <x:c r="I6" s="7">
+        <x:f>SUM(I3:I5)</x:f>
+      </x:c>
+      <x:c r="J6" s="8">
+        <x:f>IF(G6=0,"",H6/G6)</x:f>
+      </x:c>
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -1234,6 +1374,19 @@
       <x:c r="I7" s="3"/>
       <x:c r="J7" s="3"/>
       <x:c r="K7" s="3"/>
+    </x:row>
+    <x:row r="8" spans="1:11">
+      <x:c r="A8" s="3"/>
+      <x:c r="B8" s="3"/>
+      <x:c r="C8" s="3"/>
+      <x:c r="D8" s="3"/>
+      <x:c r="E8" s="3"/>
+      <x:c r="F8" s="3"/>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3"/>
+      <x:c r="I8" s="3"/>
+      <x:c r="J8" s="3"/>
+      <x:c r="K8" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -1252,7 +1405,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K8"/>
+  <x:dimension ref="A1:K9"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -1429,16 +1582,32 @@
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
-      <x:c r="A7" s="3"/>
-      <x:c r="B7" s="3"/>
-      <x:c r="C7" s="3"/>
-      <x:c r="D7" s="3"/>
-      <x:c r="E7" s="3"/>
-      <x:c r="F7" s="3"/>
-      <x:c r="G7" s="3"/>
-      <x:c r="H7" s="3"/>
-      <x:c r="I7" s="3"/>
-      <x:c r="J7" s="3"/>
+      <x:c r="A7" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B7" s="6"/>
+      <x:c r="C7" s="6"/>
+      <x:c r="D7" s="7">
+        <x:f>SUM(D3:D6)</x:f>
+      </x:c>
+      <x:c r="E7" s="7">
+        <x:f>SUM(E3:E6)</x:f>
+      </x:c>
+      <x:c r="F7" s="8">
+        <x:f>IF(D7=0,"",E7/D7)</x:f>
+      </x:c>
+      <x:c r="G7" s="7">
+        <x:f>SUM(G3:G6)</x:f>
+      </x:c>
+      <x:c r="H7" s="7">
+        <x:f>SUM(H3:H6)</x:f>
+      </x:c>
+      <x:c r="I7" s="7">
+        <x:f>SUM(I3:I6)</x:f>
+      </x:c>
+      <x:c r="J7" s="8">
+        <x:f>IF(G7=0,"",H7/G7)</x:f>
+      </x:c>
       <x:c r="K7" s="3"/>
     </x:row>
     <x:row r="8" spans="1:11">
@@ -1453,6 +1622,19 @@
       <x:c r="I8" s="3"/>
       <x:c r="J8" s="3"/>
       <x:c r="K8" s="3"/>
+    </x:row>
+    <x:row r="9" spans="1:11">
+      <x:c r="A9" s="3"/>
+      <x:c r="B9" s="3"/>
+      <x:c r="C9" s="3"/>
+      <x:c r="D9" s="3"/>
+      <x:c r="E9" s="3"/>
+      <x:c r="F9" s="3"/>
+      <x:c r="G9" s="3"/>
+      <x:c r="H9" s="3"/>
+      <x:c r="I9" s="3"/>
+      <x:c r="J9" s="3"/>
+      <x:c r="K9" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -1471,7 +1653,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K11"/>
+  <x:dimension ref="A1:K12"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -1747,16 +1929,32 @@
       <x:c r="K9" s="3"/>
     </x:row>
     <x:row r="10" spans="1:11">
-      <x:c r="A10" s="3"/>
-      <x:c r="B10" s="3"/>
-      <x:c r="C10" s="3"/>
-      <x:c r="D10" s="3"/>
-      <x:c r="E10" s="3"/>
-      <x:c r="F10" s="3"/>
-      <x:c r="G10" s="3"/>
-      <x:c r="H10" s="3"/>
-      <x:c r="I10" s="3"/>
-      <x:c r="J10" s="3"/>
+      <x:c r="A10" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B10" s="6"/>
+      <x:c r="C10" s="6"/>
+      <x:c r="D10" s="7">
+        <x:f>SUM(D3:D9)</x:f>
+      </x:c>
+      <x:c r="E10" s="7">
+        <x:f>SUM(E3:E9)</x:f>
+      </x:c>
+      <x:c r="F10" s="8">
+        <x:f>IF(D10=0,"",E10/D10)</x:f>
+      </x:c>
+      <x:c r="G10" s="7">
+        <x:f>SUM(G3:G9)</x:f>
+      </x:c>
+      <x:c r="H10" s="7">
+        <x:f>SUM(H3:H9)</x:f>
+      </x:c>
+      <x:c r="I10" s="7">
+        <x:f>SUM(I3:I9)</x:f>
+      </x:c>
+      <x:c r="J10" s="8">
+        <x:f>IF(G10=0,"",H10/G10)</x:f>
+      </x:c>
       <x:c r="K10" s="3"/>
     </x:row>
     <x:row r="11" spans="1:11">
@@ -1771,6 +1969,19 @@
       <x:c r="I11" s="3"/>
       <x:c r="J11" s="3"/>
       <x:c r="K11" s="3"/>
+    </x:row>
+    <x:row r="12" spans="1:11">
+      <x:c r="A12" s="3"/>
+      <x:c r="B12" s="3"/>
+      <x:c r="C12" s="3"/>
+      <x:c r="D12" s="3"/>
+      <x:c r="E12" s="3"/>
+      <x:c r="F12" s="3"/>
+      <x:c r="G12" s="3"/>
+      <x:c r="H12" s="3"/>
+      <x:c r="I12" s="3"/>
+      <x:c r="J12" s="3"/>
+      <x:c r="K12" s="3"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
@@ -1789,7 +2000,7 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:K7"/>
+  <x:dimension ref="A1:K8"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="11" width="16.710625" style="0" customWidth="1"/>
@@ -1797,7 +2008,7 @@
   <x:sheetData>
     <x:row r="1" spans="1:11">
       <x:c r="A1" s="1" t="s">
-        <x:v>14</x:v>
+        <x:v>15</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:11">
@@ -1933,16 +2144,32 @@
       <x:c r="K5" s="3"/>
     </x:row>
     <x:row r="6" spans="1:11">
-      <x:c r="A6" s="3"/>
-      <x:c r="B6" s="3"/>
-      <x:c r="C6" s="3"/>
-      <x:c r="D6" s="3"/>
-      <x:c r="E6" s="3"/>
-      <x:c r="F6" s="3"/>
-      <x:c r="G6" s="3"/>
-      <x:c r="H6" s="3"/>
-      <x:c r="I6" s="3"/>
-      <x:c r="J6" s="3"/>
+      <x:c r="A6" s="6" t="s">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B6" s="6"/>
+      <x:c r="C6" s="6"/>
+      <x:c r="D6" s="7">
+        <x:f>SUM(D3:D5)</x:f>
+      </x:c>
+      <x:c r="E6" s="7">
+        <x:f>SUM(E3:E5)</x:f>
+      </x:c>
+      <x:c r="F6" s="8">
+        <x:f>IF(D6=0,"",E6/D6)</x:f>
+      </x:c>
+      <x:c r="G6" s="7">
+        <x:f>SUM(G3:G5)</x:f>
+      </x:c>
+      <x:c r="H6" s="7">
+        <x:f>SUM(H3:H5)</x:f>
+      </x:c>
+      <x:c r="I6" s="7">
+        <x:f>SUM(I3:I5)</x:f>
+      </x:c>
+      <x:c r="J6" s="8">
+        <x:f>IF(G6=0,"",H6/G6)</x:f>
+      </x:c>
       <x:c r="K6" s="3"/>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -1958,6 +2185,19 @@
       <x:c r="J7" s="3"/>
       <x:c r="K7" s="3"/>
     </x:row>
+    <x:row r="8" spans="1:11">
+      <x:c r="A8" s="3"/>
+      <x:c r="B8" s="3"/>
+      <x:c r="C8" s="3"/>
+      <x:c r="D8" s="3"/>
+      <x:c r="E8" s="3"/>
+      <x:c r="F8" s="3"/>
+      <x:c r="G8" s="3"/>
+      <x:c r="H8" s="3"/>
+      <x:c r="I8" s="3"/>
+      <x:c r="J8" s="3"/>
+      <x:c r="K8" s="3"/>
+    </x:row>
   </x:sheetData>
   <x:mergeCells count="1">
     <x:mergeCell ref="A1:B1"/>

</xml_diff>